<commit_message>
New Entity Relationship Diagram uploaded.
ERD updated for accuracy.
</commit_message>
<xml_diff>
--- a/planning_docs/Entity Relationship Diagram.xlsx
+++ b/planning_docs/Entity Relationship Diagram.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1332a08b4347893b/Desktop/MSc Health Data Science/Assessment 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="262" documentId="8_{BB03E1D3-2253-4E07-811B-71B0DC0D4BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D484E30F-4259-4A4D-8503-8E1E0970D19F}"/>
+  <xr:revisionPtr revIDLastSave="269" documentId="8_{BB03E1D3-2253-4E07-811B-71B0DC0D4BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A22E073A-BC77-4B77-8BC2-D8CDE711FD17}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" activeTab="1" xr2:uid="{185AF615-FE68-4665-96DF-946565C507AA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{185AF615-FE68-4665-96DF-946565C507AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Relationships" sheetId="1" r:id="rId1"/>
@@ -43,9 +43,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="56">
   <si>
-    <t>Hospitals</t>
-  </si>
-  <si>
     <t>Doctors</t>
   </si>
   <si>
@@ -76,15 +73,9 @@
     <t>Relationships</t>
   </si>
   <si>
-    <t>One hospital &gt; many doctors, many patients</t>
-  </si>
-  <si>
     <t>Many doctors &gt; one hospital, many prescriptions</t>
   </si>
   <si>
-    <t>Many patients &gt; one hospital, many prescriptions</t>
-  </si>
-  <si>
     <t>Many prescriptions &gt; one doctor, one patient</t>
   </si>
   <si>
@@ -209,6 +200,15 @@
   </si>
   <si>
     <t>Hospital</t>
+  </si>
+  <si>
+    <t>Linked to doctor by DoctorID</t>
+  </si>
+  <si>
+    <t>One hospital &gt; many doctors</t>
+  </si>
+  <si>
+    <t>Many patients &gt; one doctor, many prescriptions</t>
   </si>
 </sst>
 </file>
@@ -878,72 +878,72 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="C2" s="2" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="2" customFormat="1" ht="60.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="C4" s="2" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -965,118 +965,118 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:9" s="7" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
       <c r="B3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>27</v>
-      </c>
       <c r="D3" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>28</v>
-      </c>
       <c r="D4" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="5" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:9" s="5" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>27</v>
-      </c>
       <c r="D7" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2"/>
       <c r="B8" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="8" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
@@ -1084,13 +1084,13 @@
     <row r="10" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>27</v>
-      </c>
       <c r="D10" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
@@ -1098,13 +1098,13 @@
     <row r="11" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
       <c r="B11" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
@@ -1112,13 +1112,13 @@
     <row r="12" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
       <c r="B12" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
@@ -1126,52 +1126,52 @@
     </row>
     <row r="13" spans="1:9" s="7" customFormat="1" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
@@ -1179,13 +1179,13 @@
     <row r="17" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2"/>
       <c r="B17" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
@@ -1215,7 +1215,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -1223,46 +1223,46 @@
     </row>
     <row r="3" spans="1:4" s="9" customFormat="1" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>51</v>
-      </c>
       <c r="D6" s="10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>